<commit_message>
Colocando o icone no executável
</commit_message>
<xml_diff>
--- a/Suprimentos.xlsx
+++ b/Suprimentos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IRISHJ00\Documents\Up\Suprimentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F888D856-6DFE-428E-9BED-D4CEF3E1BBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E9D121-0192-427A-9E59-9D7A1FB928A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{101DF58F-0805-494F-86FF-0DF45E2C3859}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="123">
   <si>
     <t>Produtos</t>
   </si>
@@ -394,6 +394,9 @@
   </si>
   <si>
     <t xml:space="preserve">Blusa feminina manga longa tamanho P </t>
+  </si>
+  <si>
+    <t>Não</t>
   </si>
 </sst>
 </file>
@@ -624,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -711,6 +714,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2619,7 +2628,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36963CDE-E660-488E-A4B2-DCAAECEBA598}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.140625" bestFit="1" customWidth="1"/>
@@ -3243,23 +3252,43 @@
       </c>
     </row>
     <row r="32" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="B32" s="26">
+      <c r="B32" s="29">
         <v>6</v>
       </c>
-      <c r="C32" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="17" t="s">
+      <c r="C32" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="30" t="s">
         <v>119</v>
       </c>
       <c r="E32" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="F32" s="15">
+      <c r="F32" s="31">
         <v>46301</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A33" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="35">
+        <v>20</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E33" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="F33" s="20">
+        <v>46303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>